<commit_message>
Add Shah to Steering Committee
</commit_message>
<xml_diff>
--- a/excell/steering_committee.xlsx
+++ b/excell/steering_committee.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MWSCAS Web Site\2026-08 MWSCAS Web Site\MWSCAS_GitHub_Beta5\MWSCAS Steering Committee\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5237FE04-D621-4DBA-9BCA-3C3143DC0C3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BB82FC7-F4A4-487C-80C7-620F0612D0BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="471" uniqueCount="355">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="361">
   <si>
     <t>LastName</t>
   </si>
@@ -1085,6 +1085,24 @@
   </si>
   <si>
     <t>Bylaws, Future Sumposia, Web Master</t>
+  </si>
+  <si>
+    <t>Shah</t>
+  </si>
+  <si>
+    <t>Sahil</t>
+  </si>
+  <si>
+    <t>University of Maryland</t>
+  </si>
+  <si>
+    <t>301-405-0772</t>
+  </si>
+  <si>
+    <t>sshah389@umd.edu</t>
+  </si>
+  <si>
+    <t>shah.jpg</t>
   </si>
 </sst>
 </file>
@@ -1436,7 +1454,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I59"/>
+  <dimension ref="A1:I60"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.7265625" customWidth="1"/>
@@ -2847,137 +2865,163 @@
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>309</v>
+        <v>355</v>
       </c>
       <c r="B55" t="s">
-        <v>310</v>
+        <v>356</v>
       </c>
       <c r="C55" t="s">
         <v>11</v>
       </c>
       <c r="D55" t="s">
-        <v>311</v>
+        <v>357</v>
       </c>
       <c r="E55" t="s">
-        <v>312</v>
-      </c>
-      <c r="F55" t="s">
-        <v>313</v>
-      </c>
-      <c r="G55" t="s">
-        <v>314</v>
+        <v>358</v>
+      </c>
+      <c r="G55" s="1" t="s">
+        <v>359</v>
       </c>
       <c r="H55" s="1" t="s">
         <v>14</v>
       </c>
       <c r="I55" t="s">
-        <v>315</v>
+        <v>360</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>316</v>
+        <v>309</v>
       </c>
       <c r="B56" t="s">
-        <v>317</v>
+        <v>310</v>
       </c>
       <c r="C56" t="s">
-        <v>354</v>
+        <v>11</v>
       </c>
       <c r="D56" t="s">
-        <v>65</v>
+        <v>311</v>
       </c>
       <c r="E56" t="s">
-        <v>318</v>
+        <v>312</v>
       </c>
       <c r="F56" t="s">
-        <v>319</v>
+        <v>313</v>
       </c>
       <c r="G56" t="s">
-        <v>320</v>
+        <v>314</v>
       </c>
       <c r="H56" s="1" t="s">
         <v>14</v>
       </c>
       <c r="I56" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>322</v>
+        <v>316</v>
       </c>
       <c r="B57" t="s">
-        <v>323</v>
+        <v>317</v>
       </c>
       <c r="C57" t="s">
-        <v>11</v>
+        <v>354</v>
       </c>
       <c r="D57" t="s">
-        <v>23</v>
+        <v>65</v>
       </c>
       <c r="E57" t="s">
-        <v>324</v>
+        <v>318</v>
+      </c>
+      <c r="F57" t="s">
+        <v>319</v>
       </c>
       <c r="G57" t="s">
-        <v>325</v>
+        <v>320</v>
       </c>
       <c r="H57" s="1" t="s">
         <v>14</v>
       </c>
       <c r="I57" t="s">
-        <v>326</v>
+        <v>321</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>336</v>
+        <v>322</v>
       </c>
       <c r="B58" t="s">
-        <v>337</v>
+        <v>323</v>
       </c>
       <c r="C58" t="s">
         <v>11</v>
       </c>
       <c r="D58" t="s">
-        <v>292</v>
+        <v>23</v>
       </c>
       <c r="E58" t="s">
-        <v>338</v>
-      </c>
-      <c r="G58" s="1" t="s">
-        <v>339</v>
+        <v>324</v>
+      </c>
+      <c r="G58" t="s">
+        <v>325</v>
       </c>
       <c r="H58" s="1" t="s">
         <v>14</v>
       </c>
       <c r="I58" t="s">
-        <v>340</v>
+        <v>326</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
+        <v>336</v>
+      </c>
+      <c r="B59" t="s">
+        <v>337</v>
+      </c>
+      <c r="C59" t="s">
+        <v>11</v>
+      </c>
+      <c r="D59" t="s">
+        <v>292</v>
+      </c>
+      <c r="E59" t="s">
+        <v>338</v>
+      </c>
+      <c r="G59" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="H59" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I59" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A60" t="s">
         <v>327</v>
       </c>
-      <c r="B59" t="s">
+      <c r="B60" t="s">
         <v>328</v>
       </c>
-      <c r="C59" t="s">
-        <v>11</v>
-      </c>
-      <c r="D59" t="s">
+      <c r="C60" t="s">
+        <v>11</v>
+      </c>
+      <c r="D60" t="s">
         <v>329</v>
       </c>
-      <c r="E59" t="s">
+      <c r="E60" t="s">
         <v>330</v>
       </c>
-      <c r="G59" t="s">
+      <c r="G60" t="s">
         <v>331</v>
       </c>
-      <c r="H59" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="I59" t="s">
+      <c r="H60" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I60" t="s">
         <v>332</v>
       </c>
     </row>
@@ -3034,17 +3078,19 @@
     <hyperlink ref="H52" r:id="rId49" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
     <hyperlink ref="H53" r:id="rId50" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
     <hyperlink ref="H54" r:id="rId51" xr:uid="{00000000-0004-0000-0000-000032000000}"/>
-    <hyperlink ref="H55" r:id="rId52" xr:uid="{00000000-0004-0000-0000-000033000000}"/>
-    <hyperlink ref="H56" r:id="rId53" xr:uid="{00000000-0004-0000-0000-000034000000}"/>
-    <hyperlink ref="H57" r:id="rId54" xr:uid="{00000000-0004-0000-0000-000035000000}"/>
-    <hyperlink ref="H59" r:id="rId55" xr:uid="{00000000-0004-0000-0000-000036000000}"/>
+    <hyperlink ref="H56" r:id="rId52" xr:uid="{00000000-0004-0000-0000-000033000000}"/>
+    <hyperlink ref="H57" r:id="rId53" xr:uid="{00000000-0004-0000-0000-000034000000}"/>
+    <hyperlink ref="H58" r:id="rId54" xr:uid="{00000000-0004-0000-0000-000035000000}"/>
+    <hyperlink ref="H60" r:id="rId55" xr:uid="{00000000-0004-0000-0000-000036000000}"/>
     <hyperlink ref="H6" r:id="rId56" xr:uid="{1528AAE4-D8AC-43A6-8202-1C14C2F4543E}"/>
-    <hyperlink ref="G58" r:id="rId57" xr:uid="{7401F541-37AB-402F-B517-5E2F4D804756}"/>
-    <hyperlink ref="H58" r:id="rId58" xr:uid="{B7ECF16E-341E-4D34-A84C-AEA63F8E0D67}"/>
+    <hyperlink ref="G59" r:id="rId57" xr:uid="{7401F541-37AB-402F-B517-5E2F4D804756}"/>
+    <hyperlink ref="H59" r:id="rId58" xr:uid="{B7ECF16E-341E-4D34-A84C-AEA63F8E0D67}"/>
     <hyperlink ref="G38" r:id="rId59" xr:uid="{11EC35A0-60DA-46F9-B3D5-DC1443C39A1A}"/>
     <hyperlink ref="H38" r:id="rId60" xr:uid="{2F48B289-2ABB-4EB8-8E8A-B0CF496AD02D}"/>
     <hyperlink ref="G7" r:id="rId61" xr:uid="{D90A5E6D-EAF8-4FA1-A7FD-59D0A0F6C5D0}"/>
     <hyperlink ref="H7" r:id="rId62" xr:uid="{4C685598-C4B2-4E9F-ADC9-41612D41B845}"/>
+    <hyperlink ref="G55" r:id="rId63" xr:uid="{AC8EC2B0-D276-406A-BAC2-F7A25AF626A3}"/>
+    <hyperlink ref="H55" r:id="rId64" xr:uid="{7EA71D21-1BD4-47D0-A613-B485B498D443}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>